<commit_message>
Group Changes and Minor Tweaks
Changed the google sheet to have a shorter share name for the Pickup location groups.
Made changes to the Default items to be in a form that uses the term Standard instead. Did not change all variable names as was worried to make a lot of changes before tomorrow.
</commit_message>
<xml_diff>
--- a/test_notebooks_R/PotPlant_File.xlsx
+++ b/test_notebooks_R/PotPlant_File.xlsx
@@ -35,7 +35,199 @@
     <t xml:space="preserve">time</t>
   </si>
   <si>
-    <t xml:space="preserve">Fair Shares Thursday Pickup</t>
+    <t xml:space="preserve">FSC-T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overberg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Basil Genovese</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mothership Pickup Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@3:30-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Chocolate Mint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Cilantro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Oregano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Parsley</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heisel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Katie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Big Boy Tomatoes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@4:30-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Jalapeno Peppers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Romaine Lettuce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Sage Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Thai Basil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vasbinder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Yarrow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schuette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melissa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Calendula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@5:30-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Rhubarb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alvarado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magdalena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Lavender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Marigolds Dwarf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Nasturtium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maggie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@4-4:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Cress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Fairy Tale Eggplant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Hyssop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hassman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lynn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant -  Sweet Red Pepper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Dill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - San Marzano Tomato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Strawberry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Sungold Tomato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Tomato Green Zebra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peeler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rataj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Tomato Super Sweet 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Zinnia Cali Mix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duello</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Marigolds Sparky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pot Plant - Zinnia Dahlia Mix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSG-Thu</t>
   </si>
   <si>
     <t xml:space="preserve">Aquilino</t>
@@ -47,211 +239,19 @@
     <t xml:space="preserve">1 Pot Plant - Angelica</t>
   </si>
   <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Shen (staff)</t>
   </si>
   <si>
     <t xml:space="preserve">Tina</t>
   </si>
   <si>
-    <t xml:space="preserve">1 Pot Plant - Basil Genovese</t>
-  </si>
-  <si>
     <t xml:space="preserve">1 Pot Plant - Holy Basil</t>
   </si>
   <si>
-    <t xml:space="preserve">1 Pot Plant - Parsley</t>
-  </si>
-  <si>
     <t xml:space="preserve">1 Pot Plant - Peppermint</t>
   </si>
   <si>
     <t xml:space="preserve">1 Pot Plant - Spearmint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSC-T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mothership Pickup Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@3:30-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Chocolate Mint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Cilantro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Oregano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heisel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Katie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Big Boy Tomatoes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@4:30-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Jalapeno Peppers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Romaine Lettuce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Sage Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Thai Basil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vasbinder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emily</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Yarrow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schuette</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melissa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Calendula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@5:30-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Rhubarb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alvarado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magdalena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Lavender</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Marigolds Dwarf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Nasturtium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Storey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maggie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@4-4:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Cress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Fairy Tale Eggplant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Hyssop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hassman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lynn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant -  Sweet Red Pepper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Dill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - San Marzano Tomato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Strawberry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Sungold Tomato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Tomato Green Zebra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peeler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rataj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Tomato Super Sweet 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Zinnia Cali Mix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duello</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Marigolds Sparky</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Pot Plant - Zinnia Dahlia Mix</t>
   </si>
   <si>
     <t xml:space="preserve">FSMini-t</t>
@@ -697,18 +697,22 @@
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2"/>
-      <c r="G2"/>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
@@ -716,117 +720,137 @@
       <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="F3"/>
-      <c r="G3"/>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4"/>
-      <c r="G4"/>
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
         <v>13</v>
       </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5"/>
-      <c r="G5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6"/>
-      <c r="G6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>
       </c>
-      <c r="F7"/>
-      <c r="G7"/>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>20</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
       <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
         <v>22</v>
-      </c>
-      <c r="G8" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
       <c r="D9" t="s">
         <v>24</v>
@@ -835,710 +859,686 @@
         <v>11</v>
       </c>
       <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s">
         <v>22</v>
-      </c>
-      <c r="G9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
       </c>
       <c r="D10" t="s">
         <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
         <v>22</v>
-      </c>
-      <c r="G10" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>19</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>20</v>
       </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s">
         <v>22</v>
-      </c>
-      <c r="G11" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
         <v>22</v>
-      </c>
-      <c r="G12" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F13" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E14" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G14" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E15" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G15" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G16" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E17" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G17" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G18" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" t="s">
         <v>41</v>
       </c>
-      <c r="D19" t="s">
-        <v>42</v>
-      </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F19" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G19" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F20" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G20" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E21" t="s">
         <v>40</v>
       </c>
-      <c r="C21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" t="s">
-        <v>44</v>
-      </c>
-      <c r="E21" t="s">
-        <v>45</v>
-      </c>
       <c r="F21" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G21" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B22" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D22" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E22" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F22" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G22" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D23" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="F23" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G23" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" t="s">
         <v>46</v>
-      </c>
-      <c r="B24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D24" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" t="s">
-        <v>26</v>
-      </c>
-      <c r="F24" t="s">
-        <v>22</v>
-      </c>
-      <c r="G24" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
         <v>46</v>
-      </c>
-      <c r="B25" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" t="s">
-        <v>48</v>
-      </c>
-      <c r="D25" t="s">
-        <v>50</v>
-      </c>
-      <c r="E25" t="s">
-        <v>26</v>
-      </c>
-      <c r="F25" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" t="s">
+        <v>48</v>
+      </c>
+      <c r="E26" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" t="s">
         <v>46</v>
-      </c>
-      <c r="B26" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D26" t="s">
-        <v>51</v>
-      </c>
-      <c r="E26" t="s">
-        <v>26</v>
-      </c>
-      <c r="F26" t="s">
-        <v>22</v>
-      </c>
-      <c r="G26" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" t="s">
         <v>46</v>
-      </c>
-      <c r="B27" t="s">
-        <v>47</v>
-      </c>
-      <c r="C27" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" t="s">
-        <v>52</v>
-      </c>
-      <c r="E27" t="s">
-        <v>49</v>
-      </c>
-      <c r="F27" t="s">
-        <v>22</v>
-      </c>
-      <c r="G27" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" t="s">
         <v>46</v>
-      </c>
-      <c r="B28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D28" t="s">
-        <v>16</v>
-      </c>
-      <c r="E28" t="s">
-        <v>26</v>
-      </c>
-      <c r="F28" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
         <v>46</v>
-      </c>
-      <c r="B29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" t="s">
-        <v>48</v>
-      </c>
-      <c r="D29" t="s">
-        <v>44</v>
-      </c>
-      <c r="E29" t="s">
-        <v>26</v>
-      </c>
-      <c r="F29" t="s">
-        <v>22</v>
-      </c>
-      <c r="G29" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" t="s">
+        <v>18</v>
+      </c>
+      <c r="E30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" t="s">
         <v>46</v>
-      </c>
-      <c r="B30" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" t="s">
-        <v>54</v>
-      </c>
-      <c r="D30" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" t="s">
         <v>46</v>
-      </c>
-      <c r="B31" t="s">
-        <v>53</v>
-      </c>
-      <c r="C31" t="s">
-        <v>54</v>
-      </c>
-      <c r="D31" t="s">
-        <v>56</v>
-      </c>
-      <c r="E31" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" t="s">
-        <v>22</v>
-      </c>
-      <c r="G31" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" t="s">
+        <v>45</v>
+      </c>
+      <c r="D32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" t="s">
         <v>46</v>
-      </c>
-      <c r="B32" t="s">
-        <v>53</v>
-      </c>
-      <c r="C32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D32" t="s">
-        <v>57</v>
-      </c>
-      <c r="E32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" t="s">
-        <v>22</v>
-      </c>
-      <c r="G32" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C33" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D33" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E33" t="s">
         <v>11</v>
       </c>
-      <c r="F33" t="s">
-        <v>22</v>
-      </c>
-      <c r="G33" t="s">
-        <v>55</v>
-      </c>
+      <c r="F33"/>
+      <c r="G33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B34" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C34" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D34" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E34" t="s">
         <v>11</v>
       </c>
-      <c r="F34" t="s">
-        <v>22</v>
-      </c>
-      <c r="G34" t="s">
-        <v>55</v>
-      </c>
+      <c r="F34"/>
+      <c r="G34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D35" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="E35" t="s">
         <v>11</v>
       </c>
-      <c r="F35" t="s">
-        <v>22</v>
-      </c>
-      <c r="G35" t="s">
-        <v>55</v>
-      </c>
+      <c r="F35"/>
+      <c r="G35"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" t="s">
+        <v>51</v>
+      </c>
+      <c r="D36" t="s">
         <v>53</v>
       </c>
-      <c r="C36" t="s">
-        <v>54</v>
-      </c>
-      <c r="D36" t="s">
-        <v>16</v>
-      </c>
       <c r="E36" t="s">
         <v>11</v>
       </c>
-      <c r="F36" t="s">
-        <v>22</v>
-      </c>
-      <c r="G36" t="s">
-        <v>55</v>
-      </c>
+      <c r="F36"/>
+      <c r="G36"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C37" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D37" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E37" t="s">
         <v>11</v>
       </c>
-      <c r="F37" t="s">
-        <v>22</v>
-      </c>
-      <c r="G37" t="s">
-        <v>55</v>
-      </c>
+      <c r="F37"/>
+      <c r="G37"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D38" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E38" t="s">
         <v>11</v>
       </c>
-      <c r="F38" t="s">
-        <v>22</v>
-      </c>
-      <c r="G38" t="s">
-        <v>55</v>
-      </c>
+      <c r="F38"/>
+      <c r="G38"/>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C39" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D39" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E39" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F39"/>
       <c r="G39"/>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C40" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D40" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="E40" t="s">
         <v>11</v>
@@ -1548,35 +1548,35 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D41" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="E41" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F41"/>
       <c r="G41"/>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B42" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C42" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D42" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E42" t="s">
         <v>11</v>
@@ -1586,16 +1586,16 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B43" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C43" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D43" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E43" t="s">
         <v>11</v>
@@ -1605,16 +1605,16 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B44" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D44" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="E44" t="s">
         <v>11</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B45" t="s">
         <v>59</v>
@@ -1633,17 +1633,21 @@
         <v>60</v>
       </c>
       <c r="D45" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E45" t="s">
-        <v>26</v>
-      </c>
-      <c r="F45"/>
-      <c r="G45"/>
+        <v>61</v>
+      </c>
+      <c r="F45" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
         <v>59</v>
@@ -1652,17 +1656,21 @@
         <v>60</v>
       </c>
       <c r="D46" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="E46" t="s">
-        <v>11</v>
-      </c>
-      <c r="F46"/>
-      <c r="G46"/>
+        <v>16</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B47" t="s">
         <v>59</v>
@@ -1671,17 +1679,21 @@
         <v>60</v>
       </c>
       <c r="D47" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="E47" t="s">
-        <v>26</v>
-      </c>
-      <c r="F47"/>
-      <c r="G47"/>
+        <v>40</v>
+      </c>
+      <c r="F47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B48" t="s">
         <v>59</v>
@@ -1690,17 +1702,21 @@
         <v>60</v>
       </c>
       <c r="D48" t="s">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="E48" t="s">
-        <v>11</v>
-      </c>
-      <c r="F48"/>
-      <c r="G48"/>
+        <v>16</v>
+      </c>
+      <c r="F48" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B49" t="s">
         <v>59</v>
@@ -1709,197 +1725,205 @@
         <v>60</v>
       </c>
       <c r="D49" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E49" t="s">
-        <v>11</v>
-      </c>
-      <c r="F49"/>
-      <c r="G49"/>
+        <v>62</v>
+      </c>
+      <c r="F49" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
+        <v>58</v>
+      </c>
+      <c r="B50" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" t="s">
         <v>46</v>
       </c>
-      <c r="B50" t="s">
-        <v>59</v>
-      </c>
-      <c r="C50" t="s">
-        <v>60</v>
-      </c>
-      <c r="D50" t="s">
-        <v>66</v>
-      </c>
-      <c r="E50" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50"/>
-      <c r="G50"/>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B51" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C51" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D51" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E51" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="F51" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G51" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B52" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C52" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D52" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E52" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F52" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G52" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B53" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C53" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D53" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="E53" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G53" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
+        <v>58</v>
+      </c>
+      <c r="B54" t="s">
         <v>67</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>68</v>
       </c>
-      <c r="C54" t="s">
-        <v>69</v>
-      </c>
       <c r="D54" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E54" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F54" t="s">
+        <v>12</v>
+      </c>
+      <c r="G54" t="s">
         <v>22</v>
-      </c>
-      <c r="G54" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
+        <v>58</v>
+      </c>
+      <c r="B55" t="s">
         <v>67</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>68</v>
       </c>
-      <c r="C55" t="s">
-        <v>69</v>
-      </c>
       <c r="D55" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="E55" t="s">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="F55" t="s">
+        <v>12</v>
+      </c>
+      <c r="G55" t="s">
         <v>22</v>
-      </c>
-      <c r="G55" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" t="s">
         <v>67</v>
       </c>
-      <c r="B56" t="s">
-        <v>72</v>
-      </c>
       <c r="C56" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D56" t="s">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E56" t="s">
         <v>11</v>
       </c>
       <c r="F56" t="s">
+        <v>12</v>
+      </c>
+      <c r="G56" t="s">
         <v>22</v>
-      </c>
-      <c r="G56" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
+        <v>58</v>
+      </c>
+      <c r="B57" t="s">
         <v>67</v>
       </c>
-      <c r="B57" t="s">
-        <v>72</v>
-      </c>
       <c r="C57" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D57" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="E57" t="s">
         <v>11</v>
       </c>
       <c r="F57" t="s">
+        <v>12</v>
+      </c>
+      <c r="G57" t="s">
         <v>22</v>
-      </c>
-      <c r="G57" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B58" t="s">
         <v>72</v>
@@ -1913,91 +1937,75 @@
       <c r="E58" t="s">
         <v>11</v>
       </c>
-      <c r="F58" t="s">
-        <v>22</v>
-      </c>
-      <c r="G58" t="s">
-        <v>55</v>
-      </c>
+      <c r="F58"/>
+      <c r="G58"/>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B59" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C59" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D59" t="s">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="E59" t="s">
         <v>11</v>
       </c>
-      <c r="F59" t="s">
-        <v>22</v>
-      </c>
-      <c r="G59" t="s">
-        <v>55</v>
-      </c>
+      <c r="F59"/>
+      <c r="G59"/>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B60" t="s">
+        <v>75</v>
+      </c>
+      <c r="C60" t="s">
         <v>76</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>77</v>
       </c>
-      <c r="D60" t="s">
-        <v>25</v>
-      </c>
       <c r="E60" t="s">
         <v>11</v>
       </c>
-      <c r="F60" t="s">
-        <v>22</v>
-      </c>
-      <c r="G60" t="s">
-        <v>31</v>
-      </c>
+      <c r="F60"/>
+      <c r="G60"/>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B61" t="s">
+        <v>75</v>
+      </c>
+      <c r="C61" t="s">
         <v>76</v>
       </c>
-      <c r="C61" t="s">
-        <v>77</v>
-      </c>
       <c r="D61" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="E61" t="s">
         <v>11</v>
       </c>
-      <c r="F61" t="s">
-        <v>22</v>
-      </c>
-      <c r="G61" t="s">
-        <v>31</v>
-      </c>
+      <c r="F61"/>
+      <c r="G61"/>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B62" t="s">
+        <v>75</v>
+      </c>
+      <c r="C62" t="s">
         <v>76</v>
-      </c>
-      <c r="C62" t="s">
-        <v>77</v>
       </c>
       <c r="D62" t="s">
         <v>78</v>
@@ -2005,22 +2013,18 @@
       <c r="E62" t="s">
         <v>11</v>
       </c>
-      <c r="F62" t="s">
-        <v>22</v>
-      </c>
-      <c r="G62" t="s">
-        <v>31</v>
-      </c>
+      <c r="F62"/>
+      <c r="G62"/>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B63" t="s">
+        <v>75</v>
+      </c>
+      <c r="C63" t="s">
         <v>76</v>
-      </c>
-      <c r="C63" t="s">
-        <v>77</v>
       </c>
       <c r="D63" t="s">
         <v>79</v>
@@ -2028,12 +2032,8 @@
       <c r="E63" t="s">
         <v>11</v>
       </c>
-      <c r="F63" t="s">
-        <v>22</v>
-      </c>
-      <c r="G63" t="s">
-        <v>31</v>
-      </c>
+      <c r="F63"/>
+      <c r="G63"/>
     </row>
     <row r="64">
       <c r="A64" t="s">
@@ -2043,16 +2043,16 @@
         <v>81</v>
       </c>
       <c r="C64" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D64" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E64" t="s">
         <v>11</v>
       </c>
       <c r="F64" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G64" t="s">
         <v>82</v>
@@ -2066,16 +2066,16 @@
         <v>81</v>
       </c>
       <c r="C65" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D65" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
       </c>
       <c r="F65" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G65" t="s">
         <v>82</v>
@@ -2089,16 +2089,16 @@
         <v>81</v>
       </c>
       <c r="C66" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D66" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="E66" t="s">
         <v>11</v>
       </c>
       <c r="F66" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G66" t="s">
         <v>82</v>
@@ -2112,16 +2112,16 @@
         <v>81</v>
       </c>
       <c r="C67" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D67" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="E67" t="s">
         <v>11</v>
       </c>
       <c r="F67" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G67" t="s">
         <v>82</v>
@@ -2135,16 +2135,16 @@
         <v>81</v>
       </c>
       <c r="C68" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D68" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="E68" t="s">
         <v>11</v>
       </c>
       <c r="F68" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G68" t="s">
         <v>82</v>
@@ -2158,16 +2158,16 @@
         <v>81</v>
       </c>
       <c r="C69" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D69" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E69" t="s">
         <v>11</v>
       </c>
       <c r="F69" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G69" t="s">
         <v>82</v>
@@ -2181,7 +2181,7 @@
         <v>81</v>
       </c>
       <c r="C70" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D70" t="s">
         <v>83</v>
@@ -2190,7 +2190,7 @@
         <v>11</v>
       </c>
       <c r="F70" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G70" t="s">
         <v>82</v>
@@ -2204,16 +2204,16 @@
         <v>81</v>
       </c>
       <c r="C71" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D71" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E71" t="s">
         <v>11</v>
       </c>
       <c r="F71" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G71" t="s">
         <v>82</v>
@@ -2227,7 +2227,7 @@
         <v>81</v>
       </c>
       <c r="C72" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D72" t="s">
         <v>84</v>
@@ -2236,7 +2236,7 @@
         <v>11</v>
       </c>
       <c r="F72" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G72" t="s">
         <v>82</v>
@@ -2250,7 +2250,7 @@
         <v>81</v>
       </c>
       <c r="C73" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D73" t="s">
         <v>85</v>
@@ -2259,7 +2259,7 @@
         <v>11</v>
       </c>
       <c r="F73" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G73" t="s">
         <v>82</v>
@@ -2276,13 +2276,13 @@
         <v>87</v>
       </c>
       <c r="D74" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E74" t="s">
         <v>11</v>
       </c>
       <c r="F74" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G74" t="s">
         <v>82</v>
@@ -2305,7 +2305,7 @@
         <v>11</v>
       </c>
       <c r="F75" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G75" t="s">
         <v>82</v>
@@ -2322,7 +2322,7 @@
         <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E76" t="s">
         <v>11</v>
@@ -2360,7 +2360,7 @@
         <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E78" t="s">
         <v>11</v>
@@ -2379,7 +2379,7 @@
         <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E79" t="s">
         <v>11</v>
@@ -2436,10 +2436,10 @@
         <v>90</v>
       </c>
       <c r="D82" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E82" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F82"/>
       <c r="G82"/>
@@ -2455,7 +2455,7 @@
         <v>90</v>
       </c>
       <c r="D83" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E83" t="s">
         <v>11</v>
@@ -2474,10 +2474,10 @@
         <v>90</v>
       </c>
       <c r="D84" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E84" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F84"/>
       <c r="G84"/>
@@ -2493,7 +2493,7 @@
         <v>96</v>
       </c>
       <c r="D85" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E85" t="s">
         <v>11</v>
@@ -2512,7 +2512,7 @@
         <v>96</v>
       </c>
       <c r="D86" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="E86" t="s">
         <v>11</v>
@@ -2531,7 +2531,7 @@
         <v>96</v>
       </c>
       <c r="D87" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E87" t="s">
         <v>11</v>
@@ -2550,10 +2550,10 @@
         <v>96</v>
       </c>
       <c r="D88" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E88" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F88"/>
       <c r="G88"/>
@@ -2569,7 +2569,7 @@
         <v>96</v>
       </c>
       <c r="D89" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="E89" t="s">
         <v>11</v>
@@ -2588,7 +2588,7 @@
         <v>96</v>
       </c>
       <c r="D90" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E90" t="s">
         <v>11</v>
@@ -2610,7 +2610,7 @@
         <v>83</v>
       </c>
       <c r="E91" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F91"/>
       <c r="G91"/>
@@ -2626,10 +2626,10 @@
         <v>98</v>
       </c>
       <c r="D92" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E92" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F92"/>
       <c r="G92"/>
@@ -2645,7 +2645,7 @@
         <v>101</v>
       </c>
       <c r="D93" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E93" t="s">
         <v>11</v>
@@ -2664,7 +2664,7 @@
         <v>101</v>
       </c>
       <c r="D94" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E94" t="s">
         <v>11</v>
@@ -2683,10 +2683,10 @@
         <v>103</v>
       </c>
       <c r="D95" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E95" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F95"/>
       <c r="G95"/>
@@ -2702,7 +2702,7 @@
         <v>105</v>
       </c>
       <c r="D96" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E96" t="s">
         <v>11</v>

</xml_diff>